<commit_message>
90% working js need to fix map sizing issue
</commit_message>
<xml_diff>
--- a/public/files/Data_By_Towns_Index/Burlington/Burlington Township.xlsx
+++ b/public/files/Data_By_Towns_Index/Burlington/Burlington Township.xlsx
@@ -428,6 +428,9 @@
       <c r="H2" t="str">
         <v>ChIJPzvlFANMwYkRRB_xOVaUkkY</v>
       </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -454,6 +457,9 @@
       <c r="H3" t="str">
         <v>ChIJl5YQFQNMwYkR3e0IowDnFhM</v>
       </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -480,6 +486,9 @@
       <c r="H4" t="str">
         <v>ChIJLXCyIgNMwYkR3-d-XJSYOWE</v>
       </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -506,6 +515,9 @@
       <c r="H5" t="str">
         <v>ChIJLXCyIgNMwYkR3-d-XJSYOWE</v>
       </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -532,6 +544,9 @@
       <c r="H6" t="str">
         <v>ChIJZc79IANMwYkR6MJeQ5a8lD4</v>
       </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -558,6 +573,9 @@
       <c r="H7" t="str">
         <v>ChIJ37qSIANMwYkRSEv4B2ajvYc</v>
       </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -584,6 +602,9 @@
       <c r="H8" t="str">
         <v>ChIJ091i2AJMwYkR9mUUmBfuzG4</v>
       </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -610,6 +631,9 @@
       <c r="H9" t="str">
         <v>ChIJd6A6FwNMwYkRVdlHCzXV8gg</v>
       </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -636,6 +660,9 @@
       <c r="H10" t="str">
         <v>ChIJd6A6FwNMwYkRVdlHCzXV8gg</v>
       </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -662,6 +689,9 @@
       <c r="H11" t="str">
         <v>ChIJwdPwHQNMwYkR_6oaOCubEAk</v>
       </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -688,6 +718,9 @@
       <c r="H12" t="str">
         <v>ChIJL9WAHANMwYkRoEONhjMY4HA</v>
       </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -714,6 +747,9 @@
       <c r="H13" t="str">
         <v>ChIJ_d3rGgNMwYkR28sr2GdDt9o</v>
       </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -740,6 +776,9 @@
       <c r="H14" t="str">
         <v>ChIJIeWuBQNMwYkRSS7PhfdixUw</v>
       </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -766,6 +805,9 @@
       <c r="H15" t="str">
         <v>ChIJ_bNYBANMwYkR_VdSsAi7-Yc</v>
       </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -792,6 +834,9 @@
       <c r="H16" t="str">
         <v>ChIJ-1pmBANMwYkRJUgNi9LAuHE</v>
       </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -818,6 +863,9 @@
       <c r="H17" t="str">
         <v>ChIJyQsvqANMwYkRcU_3intY2x8</v>
       </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -844,6 +892,9 @@
       <c r="H18" t="str">
         <v>ChIJF10-qANMwYkRX2bEBJcCm-0</v>
       </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -870,6 +921,9 @@
       <c r="H19" t="str">
         <v>ChIJ22_QoANMwYkRSHduaI7MUrw</v>
       </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -896,6 +950,9 @@
       <c r="H20" t="str">
         <v>ChIJYzCyKgNMwYkRseG0nZOIrPI</v>
       </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -922,6 +979,9 @@
       <c r="H21" t="str">
         <v>ChIJ36GCvxxMwYkRpKtAyFusZ34</v>
       </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -2224,6 +2284,9 @@
       <c r="H66" t="str">
         <v>ChIJZaW9Z71OwYkR1kJ_SqLMteo</v>
       </c>
+      <c r="I66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2250,6 +2313,9 @@
       <c r="H67" t="str">
         <v>ChIJzWlbo6JOwYkRSzYrV5GvOpg</v>
       </c>
+      <c r="I67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2276,6 +2342,9 @@
       <c r="H68" t="str">
         <v>ChIJYRqldKJOwYkR2BmAhJB6I8Q</v>
       </c>
+      <c r="I68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2302,6 +2371,9 @@
       <c r="H69" t="str">
         <v>ChIJQ7cJ-qFOwYkRbuuUHQV1O78</v>
       </c>
+      <c r="I69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2328,6 +2400,9 @@
       <c r="H70" t="str">
         <v>ChIJsT9ajh9MwYkRI0nzC6uX9Pw</v>
       </c>
+      <c r="I70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -2354,6 +2429,9 @@
       <c r="H71" t="str">
         <v>ChIJuYopKSJMwYkR2sZRIGEDJiQ</v>
       </c>
+      <c r="I71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2380,6 +2458,9 @@
       <c r="H72" t="str">
         <v>Eio1MSBDcmVla3NpZGUgV3ksIEJ1cmxpbmd0b24sIE5KIDA4MDE2LCBVU0EiMBIuChQKEglZS-wHFkzBiRENIyVRE1CNGhAzKhQKEgk9AVkkPkzBiRHrR6qnbdwpCA</v>
       </c>
+      <c r="I72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -2406,6 +2487,9 @@
       <c r="H73" t="str">
         <v>ChIJyUODBz5MwYkR6-_4TdCHiWg</v>
       </c>
+      <c r="I73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -2432,6 +2516,9 @@
       <c r="H74" t="str">
         <v>ChIJ-9KV9RVMwYkRms5VYkY_weU</v>
       </c>
+      <c r="I74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -2458,6 +2545,9 @@
       <c r="H75" t="str">
         <v>ChIJ43Cz4xVMwYkRqIGWIjCd-LY</v>
       </c>
+      <c r="I75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -2484,6 +2574,9 @@
       <c r="H76" t="str">
         <v>Eio5NiBDcmVla3NpZGUgV3ksIEJ1cmxpbmd0b24sIE5KIDA4MDE2LCBVU0EiMBIuChQKEgnNCuHqFUzBiRFlqAWgCYWx8RBgKhQKEgk9AVkkPkzBiRHrR6qnbdwpCA</v>
       </c>
+      <c r="I76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -2510,6 +2603,9 @@
       <c r="H77" t="str">
         <v>EisxMTkgQ3JlZWtzaWRlIFd5LCBCdXJsaW5ndG9uLCBOSiAwODAxNiwgVVNBIjASLgoUChIJzQrh6hVMwYkRZKgFoAmFsfEQdyoUChIJPQFZJD5MwYkR60eqp23cKQg</v>
       </c>
+      <c r="I77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -2536,6 +2632,9 @@
       <c r="H78" t="str">
         <v>ChIJFbUkohVMwYkRvNQ3I41HSTc</v>
       </c>
+      <c r="I78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -2562,6 +2661,9 @@
       <c r="H79" t="str">
         <v>ChIJSRNF7QFMwYkR-j4i41AwpiU</v>
       </c>
+      <c r="I79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -2588,6 +2690,9 @@
       <c r="H80" t="str">
         <v>ChIJ7Uu88AFMwYkR562uXJSmLRg</v>
       </c>
+      <c r="I80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -2614,6 +2719,9 @@
       <c r="H81" t="str">
         <v>ChIJoXK--QFMwYkRaHlPovRrvPY</v>
       </c>
+      <c r="I81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -2640,6 +2748,9 @@
       <c r="H82" t="str">
         <v>ChIJl_-6_wFMwYkRoeKIQyBFork</v>
       </c>
+      <c r="I82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -2666,6 +2777,9 @@
       <c r="H83" t="str">
         <v>ChIJ3Zc8_gFMwYkRHxsgiIrtpJU</v>
       </c>
+      <c r="I83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -2692,6 +2806,9 @@
       <c r="H84" t="str">
         <v>ChIJy9mt-gFMwYkRp9g2syqIIz0</v>
       </c>
+      <c r="I84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -2718,6 +2835,9 @@
       <c r="H85" t="str">
         <v>ChIJr42D6AFMwYkRoWixWeRZvs0</v>
       </c>
+      <c r="I85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -2744,6 +2864,9 @@
       <c r="H86" t="str">
         <v>ChIJG0jj3AFMwYkR0EGHoD0FFYM</v>
       </c>
+      <c r="I86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -2770,6 +2893,9 @@
       <c r="H87" t="str">
         <v>ChIJmaB9xAFMwYkRizb1UUOW_v0</v>
       </c>
+      <c r="I87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -2796,6 +2922,9 @@
       <c r="H88" t="str">
         <v>ChIJae79uQFMwYkRgDurNGFOA9E</v>
       </c>
+      <c r="I88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -2821,6 +2950,9 @@
       </c>
       <c r="H89" t="str">
         <v>ChIJjzgGugFMwYkRlZOO4OLWwRk</v>
+      </c>
+      <c r="I89" t="str">
+        <v/>
       </c>
     </row>
     <row r="90">

</xml_diff>